<commit_message>
changes in results (school as college)
</commit_message>
<xml_diff>
--- a/questiondemo.xlsx
+++ b/questiondemo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\CPF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{267145AB-24CC-4C27-8099-FDD23B8883F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7462CF5B-BFB7-4049-B1B9-850440A181BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{404EB607-DF7E-41A0-90AD-DC0CD95D3120}"/>
+    <workbookView xWindow="4248" yWindow="3540" windowWidth="17280" windowHeight="9420" xr2:uid="{404EB607-DF7E-41A0-90AD-DC0CD95D3120}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="51">
   <si>
     <t>questionnumber</t>
   </si>
@@ -45,59 +45,155 @@
     <t>category</t>
   </si>
   <si>
-    <t>I have been feeling optimistic about the future</t>
-  </si>
-  <si>
-    <t>I have been feeling useful</t>
-  </si>
-  <si>
-    <t>I have been feeling relaxed</t>
-  </si>
-  <si>
-    <t>I have been feeling interested in other people</t>
-  </si>
-  <si>
-    <t>I have been dealing with problems well</t>
-  </si>
-  <si>
-    <t>I have been thinking clearly</t>
-  </si>
-  <si>
-    <t>I have been feeling good about myself</t>
-  </si>
-  <si>
-    <t>I have been feeling close to other people</t>
-  </si>
-  <si>
-    <t>I have been feeling confident</t>
-  </si>
-  <si>
-    <t>I have been feeling loved</t>
-  </si>
-  <si>
-    <t>I have been able to make up my own mind about things</t>
-  </si>
-  <si>
-    <t>I often find it difficult to adjust my life according to the circumstances.</t>
-  </si>
-  <si>
-    <t>I have had energy to spare</t>
-  </si>
-  <si>
-    <t>I have been interested in new things</t>
-  </si>
-  <si>
-    <t>I have been feeling cheerful</t>
-  </si>
-  <si>
-    <t>Personality</t>
+    <t>I like to work on cars</t>
+  </si>
+  <si>
+    <t>I like to do puzzles</t>
+  </si>
+  <si>
+    <t>I am good at working independently</t>
+  </si>
+  <si>
+    <t>I like to work in teams</t>
+  </si>
+  <si>
+    <t>I am an ambitious person, I set goals for myself</t>
+  </si>
+  <si>
+    <t>I like to organize things (files, desks/offices)</t>
+  </si>
+  <si>
+    <t>I like to build things</t>
+  </si>
+  <si>
+    <t>I like to read about art and music</t>
+  </si>
+  <si>
+    <t>I like to have clear instructions to follow</t>
+  </si>
+  <si>
+    <t>I like to try to influence or persuade people</t>
+  </si>
+  <si>
+    <t>I like to do experiments</t>
+  </si>
+  <si>
+    <t>I like to teach or train people</t>
+  </si>
+  <si>
+    <t>I like trying to help people solve their problems</t>
+  </si>
+  <si>
+    <t>I like to take care of animals</t>
+  </si>
+  <si>
+    <t>I wouldn’t mind working 8 hours per day in an office</t>
+  </si>
+  <si>
+    <t>I like selling things</t>
+  </si>
+  <si>
+    <t>I enjoy creative writing</t>
+  </si>
+  <si>
+    <t>I enjoy science</t>
+  </si>
+  <si>
+    <t>I am quick to take on new responsibilities</t>
+  </si>
+  <si>
+    <t>I am interested in healing people</t>
+  </si>
+  <si>
+    <t>I enjoy trying to figure out how things work</t>
+  </si>
+  <si>
+    <t>I like putting things together or assembling things</t>
+  </si>
+  <si>
+    <t>I am a creative person</t>
+  </si>
+  <si>
+    <t>I pay attention to details</t>
+  </si>
+  <si>
+    <t>I like to do filing or typing</t>
+  </si>
+  <si>
+    <t>I like to analyze things (problems/situations)</t>
+  </si>
+  <si>
+    <t>I like to play instruments or sing</t>
+  </si>
+  <si>
+    <t>I enjoy learning about other cultures</t>
+  </si>
+  <si>
+    <t>I would like to start my own business</t>
+  </si>
+  <si>
+    <t>I like to cook</t>
+  </si>
+  <si>
+    <t>I like acting in plays</t>
+  </si>
+  <si>
+    <t>I am a practical person</t>
+  </si>
+  <si>
+    <t>I like working with numbers or charts</t>
+  </si>
+  <si>
+    <t>I like to get into discussions about issues</t>
+  </si>
+  <si>
+    <t>I am good at keeping records of my work</t>
+  </si>
+  <si>
+    <t>I like to lead</t>
+  </si>
+  <si>
+    <t>I like working outdoors</t>
+  </si>
+  <si>
+    <t>I would like to work in an office</t>
+  </si>
+  <si>
+    <t>I’m good at math</t>
+  </si>
+  <si>
+    <t>I like helping people</t>
+  </si>
+  <si>
+    <t>I like to draw</t>
+  </si>
+  <si>
+    <t>I like to give speeches</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>C</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -105,26 +201,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="7"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -139,12 +222,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -459,7 +541,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E806D458-456B-4FBA-9955-7D4F7BC4D43A}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -473,59 +555,59 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="C2" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="C3" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="C4" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="C5" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>18</v>
+        <v>7</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
@@ -533,32 +615,32 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>18</v>
+        <v>10</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
@@ -566,32 +648,32 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>18</v>
+      <c r="C12" s="1" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
@@ -599,21 +681,21 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
@@ -621,21 +703,318 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A17" s="1">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>18</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A18" s="1">
+        <v>17</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="1">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A20" s="1">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+      <c r="A21" s="1">
+        <v>20</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A22" s="1">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="1">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A24" s="1">
+        <v>23</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A25" s="1">
+        <v>24</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A26" s="1">
+        <v>25</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A27" s="1">
+        <v>26</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+      <c r="A28" s="1">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+      <c r="A29" s="1">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+      <c r="A30" s="1">
+        <v>29</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A31" s="1">
+        <v>30</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A32" s="1">
+        <v>31</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A33" s="1">
+        <v>32</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+      <c r="A34" s="1">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+      <c r="A35" s="1">
+        <v>34</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A36" s="1">
+        <v>35</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A37" s="1">
+        <v>36</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A38" s="1">
+        <v>37</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A39" s="1">
+        <v>38</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A40" s="1">
+        <v>39</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A41" s="1">
+        <v>40</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A42" s="1">
+        <v>41</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A43" s="1">
+        <v>42</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
name and new sets are added
</commit_message>
<xml_diff>
--- a/questiondemo.xlsx
+++ b/questiondemo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\CPF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7462CF5B-BFB7-4049-B1B9-850440A181BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDB38250-307E-4B18-BA46-5A963F619A88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4248" yWindow="3540" windowWidth="17280" windowHeight="9420" xr2:uid="{404EB607-DF7E-41A0-90AD-DC0CD95D3120}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{404EB607-DF7E-41A0-90AD-DC0CD95D3120}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="49">
   <si>
     <t>questionnumber</t>
   </si>
@@ -45,148 +45,142 @@
     <t>category</t>
   </si>
   <si>
-    <t>I like to work on cars</t>
-  </si>
-  <si>
-    <t>I like to do puzzles</t>
-  </si>
-  <si>
-    <t>I am good at working independently</t>
-  </si>
-  <si>
-    <t>I like to work in teams</t>
-  </si>
-  <si>
-    <t>I am an ambitious person, I set goals for myself</t>
-  </si>
-  <si>
-    <t>I like to organize things (files, desks/offices)</t>
-  </si>
-  <si>
-    <t>I like to build things</t>
-  </si>
-  <si>
-    <t>I like to read about art and music</t>
-  </si>
-  <si>
-    <t>I like to have clear instructions to follow</t>
-  </si>
-  <si>
-    <t>I like to try to influence or persuade people</t>
-  </si>
-  <si>
-    <t>I like to do experiments</t>
-  </si>
-  <si>
-    <t>I like to teach or train people</t>
-  </si>
-  <si>
-    <t>I like trying to help people solve their problems</t>
-  </si>
-  <si>
-    <t>I like to take care of animals</t>
-  </si>
-  <si>
-    <t>I wouldn’t mind working 8 hours per day in an office</t>
-  </si>
-  <si>
-    <t>I like selling things</t>
-  </si>
-  <si>
-    <t>I enjoy creative writing</t>
-  </si>
-  <si>
-    <t>I enjoy science</t>
-  </si>
-  <si>
-    <t>I am quick to take on new responsibilities</t>
-  </si>
-  <si>
-    <t>I am interested in healing people</t>
-  </si>
-  <si>
-    <t>I enjoy trying to figure out how things work</t>
-  </si>
-  <si>
-    <t>I like putting things together or assembling things</t>
-  </si>
-  <si>
-    <t>I am a creative person</t>
-  </si>
-  <si>
-    <t>I pay attention to details</t>
-  </si>
-  <si>
-    <t>I like to do filing or typing</t>
-  </si>
-  <si>
-    <t>I like to analyze things (problems/situations)</t>
-  </si>
-  <si>
-    <t>I like to play instruments or sing</t>
-  </si>
-  <si>
-    <t>I enjoy learning about other cultures</t>
-  </si>
-  <si>
-    <t>I would like to start my own business</t>
-  </si>
-  <si>
-    <t>I like to cook</t>
-  </si>
-  <si>
-    <t>I like acting in plays</t>
-  </si>
-  <si>
-    <t>I am a practical person</t>
-  </si>
-  <si>
-    <t>I like working with numbers or charts</t>
-  </si>
-  <si>
-    <t>I like to get into discussions about issues</t>
-  </si>
-  <si>
-    <t>I am good at keeping records of my work</t>
-  </si>
-  <si>
-    <t>I like to lead</t>
-  </si>
-  <si>
-    <t>I like working outdoors</t>
-  </si>
-  <si>
-    <t>I would like to work in an office</t>
-  </si>
-  <si>
-    <t>I’m good at math</t>
-  </si>
-  <si>
-    <t>I like helping people</t>
-  </si>
-  <si>
-    <t>I like to draw</t>
-  </si>
-  <si>
-    <t>I like to give speeches</t>
-  </si>
-  <si>
-    <t>R</t>
-  </si>
-  <si>
-    <t>I</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>S</t>
-  </si>
-  <si>
-    <t>E</t>
-  </si>
-  <si>
-    <t>C</t>
+    <t>At home, there is an adult who is interested in my college work</t>
+  </si>
+  <si>
+    <t>Home</t>
+  </si>
+  <si>
+    <t>At home, there is an adult who believes that I will be a success</t>
+  </si>
+  <si>
+    <t>At home, there is an adult who wants me to do my best</t>
+  </si>
+  <si>
+    <t>At home, there is an adult who listens to me when I have something to say</t>
+  </si>
+  <si>
+    <t>At college, there is an adult who really cares about me</t>
+  </si>
+  <si>
+    <t>College</t>
+  </si>
+  <si>
+    <t>At college, there is an adult who tells me when I do a good job</t>
+  </si>
+  <si>
+    <t>At college, there is an adult who listens to me when I have something to say</t>
+  </si>
+  <si>
+    <t>At college, there is an adult who believes that I will be a success</t>
+  </si>
+  <si>
+    <t>Away from college, there is an adult who really cares about me</t>
+  </si>
+  <si>
+    <t>Community</t>
+  </si>
+  <si>
+    <t>Away from college, there is an adult who tells me when I do a good job</t>
+  </si>
+  <si>
+    <t>Away from college, there is an adult who believes that I will be a success</t>
+  </si>
+  <si>
+    <t>Away from college, there is an adult whom I trust</t>
+  </si>
+  <si>
+    <t>Away from college, I am a member of a club, sports team, temple association, or other group</t>
+  </si>
+  <si>
+    <t>Involvement</t>
+  </si>
+  <si>
+    <t>Away from college, I take lessons in music, art, sports, or have a hobby</t>
+  </si>
+  <si>
+    <t>Students at my college would choose me on their team</t>
+  </si>
+  <si>
+    <t>Students at my college would explain the rules of a game if I didn’t understand them</t>
+  </si>
+  <si>
+    <t>Students at my college would invite me to their home</t>
+  </si>
+  <si>
+    <t>Students at my college would share things with me</t>
+  </si>
+  <si>
+    <t>Students at my college would help me if I hurt myself</t>
+  </si>
+  <si>
+    <t>Students at my college would miss me if I wasn’t at college</t>
+  </si>
+  <si>
+    <t>Students at my college would make me feel better if something is bothering me</t>
+  </si>
+  <si>
+    <t>Students at my college would pick me for a partner</t>
+  </si>
+  <si>
+    <t>Students at my college would help me if other students are being mean to me</t>
+  </si>
+  <si>
+    <t>Students at my college would tell me I’m their friend</t>
+  </si>
+  <si>
+    <t>Students at my college would ask me to join in when I am alone</t>
+  </si>
+  <si>
+    <t>Students at my college would tell me secrets</t>
+  </si>
+  <si>
+    <t>I do things at home that make a difference (make things better)</t>
+  </si>
+  <si>
+    <t>Self</t>
+  </si>
+  <si>
+    <t>I help my family make decisions</t>
+  </si>
+  <si>
+    <t>At college, I decide things like class activities or rules</t>
+  </si>
+  <si>
+    <t>I do things at college that make a difference (make things better)</t>
+  </si>
+  <si>
+    <t>I can work out my problems</t>
+  </si>
+  <si>
+    <t>I can do most things if I try</t>
+  </si>
+  <si>
+    <t>There are many things that I do well</t>
+  </si>
+  <si>
+    <t>I feel bad when someone gets their feelings hurt</t>
+  </si>
+  <si>
+    <t>I try to understand what other people feel</t>
+  </si>
+  <si>
+    <t>When I need help, I find someone to talk to</t>
+  </si>
+  <si>
+    <t>I know where to go for help when I have a problem</t>
+  </si>
+  <si>
+    <t>I try to work out problems by talking about them</t>
+  </si>
+  <si>
+    <t>I have goals and plans for the future</t>
+  </si>
+  <si>
+    <t>I think I will be successful when I grow up</t>
+  </si>
+  <si>
+    <t>Peers</t>
   </si>
 </sst>
 </file>
@@ -555,7 +549,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -563,227 +557,227 @@
         <v>3</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="144" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="144" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:3" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="144" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
@@ -791,43 +785,43 @@
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="144" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
@@ -835,76 +829,76 @@
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="72" x14ac:dyDescent="0.3">
@@ -912,21 +906,21 @@
         <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
@@ -934,88 +928,76 @@
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A42" s="1">
-        <v>41</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A43" s="1">
-        <v>42</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>49</v>
-      </c>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="1"/>
+      <c r="B42" s="1"/>
+      <c r="C42" s="1"/>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="1"/>
+      <c r="B43" s="1"/>
+      <c r="C43" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
name changes of the domain
</commit_message>
<xml_diff>
--- a/questiondemo.xlsx
+++ b/questiondemo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\CPF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDB38250-307E-4B18-BA46-5A963F619A88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{432A4EC2-306A-4417-81BE-5BD0D25DB6CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{404EB607-DF7E-41A0-90AD-DC0CD95D3120}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="37">
   <si>
     <t>questionnumber</t>
   </si>
@@ -45,142 +45,106 @@
     <t>category</t>
   </si>
   <si>
-    <t>At home, there is an adult who is interested in my college work</t>
-  </si>
-  <si>
-    <t>Home</t>
-  </si>
-  <si>
-    <t>At home, there is an adult who believes that I will be a success</t>
-  </si>
-  <si>
-    <t>At home, there is an adult who wants me to do my best</t>
-  </si>
-  <si>
-    <t>At home, there is an adult who listens to me when I have something to say</t>
-  </si>
-  <si>
-    <t>At college, there is an adult who really cares about me</t>
-  </si>
-  <si>
-    <t>College</t>
-  </si>
-  <si>
-    <t>At college, there is an adult who tells me when I do a good job</t>
-  </si>
-  <si>
-    <t>At college, there is an adult who listens to me when I have something to say</t>
-  </si>
-  <si>
-    <t>At college, there is an adult who believes that I will be a success</t>
-  </si>
-  <si>
-    <t>Away from college, there is an adult who really cares about me</t>
-  </si>
-  <si>
-    <t>Community</t>
-  </si>
-  <si>
-    <t>Away from college, there is an adult who tells me when I do a good job</t>
-  </si>
-  <si>
-    <t>Away from college, there is an adult who believes that I will be a success</t>
-  </si>
-  <si>
-    <t>Away from college, there is an adult whom I trust</t>
-  </si>
-  <si>
-    <t>Away from college, I am a member of a club, sports team, temple association, or other group</t>
-  </si>
-  <si>
-    <t>Involvement</t>
-  </si>
-  <si>
-    <t>Away from college, I take lessons in music, art, sports, or have a hobby</t>
-  </si>
-  <si>
-    <t>Students at my college would choose me on their team</t>
-  </si>
-  <si>
-    <t>Students at my college would explain the rules of a game if I didn’t understand them</t>
-  </si>
-  <si>
-    <t>Students at my college would invite me to their home</t>
-  </si>
-  <si>
-    <t>Students at my college would share things with me</t>
-  </si>
-  <si>
-    <t>Students at my college would help me if I hurt myself</t>
-  </si>
-  <si>
-    <t>Students at my college would miss me if I wasn’t at college</t>
-  </si>
-  <si>
-    <t>Students at my college would make me feel better if something is bothering me</t>
-  </si>
-  <si>
-    <t>Students at my college would pick me for a partner</t>
-  </si>
-  <si>
-    <t>Students at my college would help me if other students are being mean to me</t>
-  </si>
-  <si>
-    <t>Students at my college would tell me I’m their friend</t>
-  </si>
-  <si>
-    <t>Students at my college would ask me to join in when I am alone</t>
-  </si>
-  <si>
-    <t>Students at my college would tell me secrets</t>
-  </si>
-  <si>
-    <t>I do things at home that make a difference (make things better)</t>
-  </si>
-  <si>
-    <t>Self</t>
-  </si>
-  <si>
-    <t>I help my family make decisions</t>
-  </si>
-  <si>
-    <t>At college, I decide things like class activities or rules</t>
-  </si>
-  <si>
-    <t>I do things at college that make a difference (make things better)</t>
-  </si>
-  <si>
-    <t>I can work out my problems</t>
-  </si>
-  <si>
-    <t>I can do most things if I try</t>
-  </si>
-  <si>
-    <t>There are many things that I do well</t>
-  </si>
-  <si>
-    <t>I feel bad when someone gets their feelings hurt</t>
-  </si>
-  <si>
-    <t>I try to understand what other people feel</t>
-  </si>
-  <si>
-    <t>When I need help, I find someone to talk to</t>
-  </si>
-  <si>
-    <t>I know where to go for help when I have a problem</t>
-  </si>
-  <si>
-    <t>I try to work out problems by talking about them</t>
-  </si>
-  <si>
-    <t>I have goals and plans for the future</t>
-  </si>
-  <si>
-    <t>I think I will be successful when I grow up</t>
-  </si>
-  <si>
-    <t>Peers</t>
+    <t>Expressing my emotions with words is not a problem for me.</t>
+  </si>
+  <si>
+    <t>Emotionality</t>
+  </si>
+  <si>
+    <t>I often find it difficult to see things from another person’s viewpoint.</t>
+  </si>
+  <si>
+    <t>On the whole, I’m a highly motivated person.</t>
+  </si>
+  <si>
+    <t>Self-Control</t>
+  </si>
+  <si>
+    <t>I usually find it difficult to regulate my emotions.</t>
+  </si>
+  <si>
+    <t>I generally don’t find life enjoyable.</t>
+  </si>
+  <si>
+    <t>Well-Being</t>
+  </si>
+  <si>
+    <t>I can deal effectively with people.</t>
+  </si>
+  <si>
+    <t>Sociability</t>
+  </si>
+  <si>
+    <t>I tend to change my mind frequently.</t>
+  </si>
+  <si>
+    <t>Many times, I can’t figure out what emotion I'm feeling.</t>
+  </si>
+  <si>
+    <t>I feel that I have a number of good qualities.</t>
+  </si>
+  <si>
+    <t>I often find it difficult to stand up for my rights.</t>
+  </si>
+  <si>
+    <t>I’m usually able to influence the way other people feel.</t>
+  </si>
+  <si>
+    <t>On the whole, I have a gloomy perspective on most things.</t>
+  </si>
+  <si>
+    <t>Those close to me often complain that I don’t treat them right.</t>
+  </si>
+  <si>
+    <t>I often find it difficult to adjust my life according to the circumstances.</t>
+  </si>
+  <si>
+    <t>On the whole, I’m able to deal with stress.</t>
+  </si>
+  <si>
+    <t>I often find it difficult to show my affection to those close to me.</t>
+  </si>
+  <si>
+    <t>I’m normally able to “get into someone’s shoes” and experience their emotions.</t>
+  </si>
+  <si>
+    <t>I normally find it difficult to keep myself motivated.</t>
+  </si>
+  <si>
+    <t>I’m usually able to find ways to control my emotions when I want to.</t>
+  </si>
+  <si>
+    <t>On the whole, I’m pleased with my life.</t>
+  </si>
+  <si>
+    <t>I would describe myself as a good negotiator.</t>
+  </si>
+  <si>
+    <t>I tend to get involved in things I later wish I could get out of.</t>
+  </si>
+  <si>
+    <t>I often pause and think about my feelings.</t>
+  </si>
+  <si>
+    <t>I believe I’m full of personal strengths.</t>
+  </si>
+  <si>
+    <t>I tend to “back down” even if I know I’m right.</t>
+  </si>
+  <si>
+    <t>I don’t seem to have any power at all over other people’s feelings.</t>
+  </si>
+  <si>
+    <t>I generally believe that things will work out fine in my life.</t>
+  </si>
+  <si>
+    <t>I find it difficult to bond well even with those close to me.</t>
+  </si>
+  <si>
+    <t>Generally, I’m able to adapt to new environments.</t>
+  </si>
+  <si>
+    <t>Others admire me for being relaxed.</t>
   </si>
 </sst>
 </file>
@@ -560,7 +524,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="144" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -571,7 +535,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -579,120 +543,120 @@
         <v>6</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="144" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="144" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="187.2" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="144" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -700,10 +664,10 @@
         <v>20</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -711,10 +675,10 @@
         <v>21</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="158.4" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -722,10 +686,10 @@
         <v>22</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -733,10 +697,10 @@
         <v>23</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -744,10 +708,10 @@
         <v>24</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="144" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -755,10 +719,10 @@
         <v>25</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -766,10 +730,10 @@
         <v>26</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="158.4" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -777,10 +741,10 @@
         <v>27</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -788,10 +752,10 @@
         <v>28</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="144" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -799,10 +763,10 @@
         <v>29</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -810,10 +774,10 @@
         <v>30</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -821,10 +785,10 @@
         <v>31</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -832,10 +796,10 @@
         <v>32</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -843,151 +807,91 @@
         <v>33</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="72" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="1">
-        <v>31</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="1">
-        <v>32</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="72" x14ac:dyDescent="0.3">
-      <c r="A34" s="1">
-        <v>33</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A35" s="1">
-        <v>34</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A36" s="1">
-        <v>35</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A37" s="1">
-        <v>36</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A38" s="1">
-        <v>37</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A39" s="1">
-        <v>38</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="72" x14ac:dyDescent="0.3">
-      <c r="A40" s="1">
-        <v>39</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" ht="72" x14ac:dyDescent="0.3">
-      <c r="A41" s="1">
-        <v>40</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>34</v>
-      </c>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="1"/>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="1"/>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="1"/>
+      <c r="B36" s="1"/>
+      <c r="C36" s="1"/>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="1"/>
+      <c r="B37" s="1"/>
+      <c r="C37" s="1"/>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="1"/>
+      <c r="B38" s="1"/>
+      <c r="C38" s="1"/>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="1"/>
+      <c r="B39" s="1"/>
+      <c r="C39" s="1"/>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="1"/>
+      <c r="B40" s="1"/>
+      <c r="C40" s="1"/>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="1"/>
+      <c r="B41" s="1"/>
+      <c r="C41" s="1"/>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>

</xml_diff>